<commit_message>
Execution of test cases
</commit_message>
<xml_diff>
--- a/Admin Module/04_Test_Execution.xlsx
+++ b/Admin Module/04_Test_Execution.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Execution ID</t>
   </si>
@@ -63,6 +63,39 @@
   </si>
   <si>
     <t>Remarks</t>
+  </si>
+  <si>
+    <t>EX-001</t>
+  </si>
+  <si>
+    <t>TC-001</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Verify Login page loads successfully</t>
+  </si>
+  <si>
+    <t>Login page should load successfully</t>
+  </si>
+  <si>
+    <t>Login page displayed</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Ahsan Mehmood</t>
+  </si>
+  <si>
+    <t>Test case passed</t>
   </si>
 </sst>
 </file>
@@ -686,12 +719,18 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1226,24 +1265,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="19.8888888888889" customWidth="1"/>
     <col min="2" max="2" width="17.8888888888889" customWidth="1"/>
     <col min="3" max="3" width="19.5555555555556" customWidth="1"/>
     <col min="4" max="4" width="18.2222222222222" customWidth="1"/>
     <col min="5" max="5" width="19.1111111111111" customWidth="1"/>
-    <col min="6" max="6" width="17.1111111111111" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="16.5555555555556" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="9" width="14.5555555555556" customWidth="1"/>
     <col min="10" max="10" width="15.4444444444444" customWidth="1"/>
     <col min="11" max="11" width="14.3333333333333" customWidth="1"/>
-    <col min="12" max="12" width="15.1111111111111" customWidth="1"/>
+    <col min="12" max="12" width="17.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.8" spans="1:12">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1279,6 +1318,44 @@
       </c>
       <c r="L1" s="1" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="2" ht="28.8" spans="1:12">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="3">
+        <v>46030</v>
+      </c>
+      <c r="L2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>